<commit_message>
Nordic comparisons follow the dissertation (Norway omitted); final reviews
- both table scripts read the dissertation's Nordic aggregate (Denmark, Finland, Iceland,
  Sweden; workbook series NoNoNordics), as in Klimantas 2025 ch. 4; notes say why Norway is omitted
- regenerated Estonia T5, Latvia T7/T8 and the Nordic macros; Lithuania now 56 -> 66 per cent
  of the Nordic average 1913-2023, as in the dissertation
- Latvia text: "only Lithuania has improved on its 1913 position" (sec. 5, conclusion)
- PDFs and Word files rebuilt
- quality_reports: final referee and domain reviews of both papers, cancelled comparator
  rebuild plan (comparators are the dissertation's own MPD 2023 data), session log

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012jmLy3YN7WhP457s5taGEh
</commit_message>
<xml_diff>
--- a/Paper/latvia/supplementary/Latvia_online_data_appendix.xlsx
+++ b/Paper/latvia/supplementary/Latvia_online_data_appendix.xlsx
@@ -10470,7 +10470,7 @@
         <v>2.15</v>
       </c>
       <c r="G2" t="n">
-        <v>1.93</v>
+        <v>1.96</v>
       </c>
       <c r="H2" t="n">
         <v>1.02</v>
@@ -10505,7 +10505,7 @@
         <v>1.59</v>
       </c>
       <c r="G3" t="n">
-        <v>1.84</v>
+        <v>1.91</v>
       </c>
       <c r="H3" t="n">
         <v>0.99</v>
@@ -10540,7 +10540,7 @@
         <v>3.14</v>
       </c>
       <c r="G4" t="n">
-        <v>2.09</v>
+        <v>2.06</v>
       </c>
       <c r="H4" t="n">
         <v>1.06</v>
@@ -10575,7 +10575,7 @@
         <v>3.09</v>
       </c>
       <c r="G5" t="n">
-        <v>2.64</v>
+        <v>2.59</v>
       </c>
       <c r="H5" t="n">
         <v>2.4</v>
@@ -10610,7 +10610,7 @@
         <v>1.42</v>
       </c>
       <c r="G6" t="n">
-        <v>2.11</v>
+        <v>2.12</v>
       </c>
       <c r="H6" t="n">
         <v>0.63</v>
@@ -10645,7 +10645,7 @@
         <v>3.64</v>
       </c>
       <c r="G7" t="n">
-        <v>3.14</v>
+        <v>3.13</v>
       </c>
       <c r="H7" t="n">
         <v>3.61</v>
@@ -10680,7 +10680,7 @@
         <v>3.58</v>
       </c>
       <c r="G8" t="n">
-        <v>2.52</v>
+        <v>2.4</v>
       </c>
       <c r="H8" t="n">
         <v>2.39</v>
@@ -10715,7 +10715,7 @@
         <v>1.17</v>
       </c>
       <c r="G9" t="n">
-        <v>1.96</v>
+        <v>1.48</v>
       </c>
       <c r="H9" t="n">
         <v>1.38</v>
@@ -10750,7 +10750,7 @@
         <v>-0.79</v>
       </c>
       <c r="G10" t="n">
-        <v>1.64</v>
+        <v>0.62</v>
       </c>
       <c r="H10" t="n">
         <v>1.34</v>
@@ -10785,7 +10785,7 @@
         <v>3.73</v>
       </c>
       <c r="G11" t="n">
-        <v>3.77</v>
+        <v>3.18</v>
       </c>
       <c r="H11" t="n">
         <v>2.41</v>
@@ -10820,7 +10820,7 @@
         <v>0.01</v>
       </c>
       <c r="G12" t="n">
-        <v>0.73</v>
+        <v>0.56</v>
       </c>
       <c r="H12" t="n">
         <v>0.62</v>
@@ -10855,7 +10855,7 @@
         <v>2.28</v>
       </c>
       <c r="G13" t="n">
-        <v>2.27</v>
+        <v>2.1</v>
       </c>
       <c r="H13" t="n">
         <v>1.77</v>
@@ -10928,13 +10928,13 @@
         <v>39</v>
       </c>
       <c r="H17" t="n">
-        <v>81.2</v>
+        <v>80.4</v>
       </c>
       <c r="I17" t="n">
-        <v>56.2</v>
+        <v>55.6</v>
       </c>
       <c r="J17" t="n">
-        <v>70.8</v>
+        <v>70.1</v>
       </c>
       <c r="K17"/>
     </row>
@@ -10961,13 +10961,13 @@
         <v>40.7</v>
       </c>
       <c r="H18" t="n">
-        <v>60.5</v>
+        <v>59.2</v>
       </c>
       <c r="I18" t="n">
-        <v>40.6</v>
+        <v>39.7</v>
       </c>
       <c r="J18" t="n">
-        <v>54.3</v>
+        <v>53.2</v>
       </c>
       <c r="K18"/>
     </row>
@@ -10994,13 +10994,13 @@
         <v>37.2</v>
       </c>
       <c r="H19" t="n">
-        <v>66.2</v>
+        <v>64.9</v>
       </c>
       <c r="I19" t="n">
-        <v>43.9</v>
+        <v>43.1</v>
       </c>
       <c r="J19" t="n">
-        <v>57.3</v>
+        <v>56.3</v>
       </c>
       <c r="K19" t="n">
         <v>144.1</v>
@@ -11029,13 +11029,13 @@
         <v>37.8</v>
       </c>
       <c r="H20" t="n">
-        <v>61.9</v>
+        <v>60.6</v>
       </c>
       <c r="I20" t="n">
-        <v>38.2</v>
+        <v>37.5</v>
       </c>
       <c r="J20" t="n">
-        <v>61</v>
+        <v>59.8</v>
       </c>
       <c r="K20" t="n">
         <v>143.9</v>
@@ -11064,13 +11064,13 @@
         <v>39.7</v>
       </c>
       <c r="H21" t="n">
-        <v>71.9</v>
+        <v>70.6</v>
       </c>
       <c r="I21" t="n">
-        <v>51.5</v>
+        <v>50.5</v>
       </c>
       <c r="J21" t="n">
-        <v>70.1</v>
+        <v>68.7</v>
       </c>
       <c r="K21" t="n">
         <v>159.3</v>
@@ -11099,13 +11099,13 @@
         <v>39.8</v>
       </c>
       <c r="H22" t="n">
-        <v>67.2</v>
+        <v>65.7</v>
       </c>
       <c r="I22" t="n">
-        <v>51</v>
+        <v>49.8</v>
       </c>
       <c r="J22" t="n">
-        <v>63.7</v>
+        <v>62.3</v>
       </c>
       <c r="K22" t="n">
         <v>154.5</v>
@@ -11134,13 +11134,13 @@
         <v>34.6</v>
       </c>
       <c r="H23" t="n">
-        <v>49.6</v>
+        <v>49.9</v>
       </c>
       <c r="I23" t="n">
-        <v>44.4</v>
+        <v>44.7</v>
       </c>
       <c r="J23" t="n">
-        <v>50.7</v>
+        <v>51</v>
       </c>
       <c r="K23" t="n">
         <v>135.5</v>
@@ -11169,13 +11169,13 @@
         <v>29</v>
       </c>
       <c r="H24" t="n">
-        <v>25.7</v>
+        <v>27.5</v>
       </c>
       <c r="I24" t="n">
-        <v>26.7</v>
+        <v>28.5</v>
       </c>
       <c r="J24" t="n">
-        <v>32.2</v>
+        <v>34.4</v>
       </c>
       <c r="K24"/>
     </row>
@@ -11202,13 +11202,13 @@
         <v>44.7</v>
       </c>
       <c r="H25" t="n">
-        <v>42.6</v>
+        <v>49.2</v>
       </c>
       <c r="I25" t="n">
-        <v>42.9</v>
+        <v>49.5</v>
       </c>
       <c r="J25" t="n">
-        <v>47.8</v>
+        <v>55.2</v>
       </c>
       <c r="K25"/>
     </row>
@@ -11235,13 +11235,13 @@
         <v>57.4</v>
       </c>
       <c r="H26" t="n">
-        <v>49.1</v>
+        <v>57.8</v>
       </c>
       <c r="I26" t="n">
-        <v>55.1</v>
+        <v>64.8</v>
       </c>
       <c r="J26" t="n">
-        <v>54.1</v>
+        <v>63.7</v>
       </c>
       <c r="K26"/>
     </row>
@@ -11268,13 +11268,13 @@
         <v>63.4</v>
       </c>
       <c r="H27" t="n">
-        <v>51.5</v>
+        <v>60.7</v>
       </c>
       <c r="I27" t="n">
-        <v>56.1</v>
+        <v>66</v>
       </c>
       <c r="J27" t="n">
-        <v>52.2</v>
+        <v>61.5</v>
       </c>
       <c r="K27"/>
     </row>

</xml_diff>